<commit_message>
Nuevos ajustes en el .exe
</commit_message>
<xml_diff>
--- a/.exe/Bot Descargas.xlsx
+++ b/.exe/Bot Descargas.xlsx
@@ -196,8 +196,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Q10_Filtros" displayName="Q10_Filtros" ref="I5:M10" headerRowCount="1">
-  <autoFilter ref="I5:M10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Q10_Filtros" displayName="Q10_Filtros" ref="I5:M12" headerRowCount="1">
+  <autoFilter ref="I5:M12"/>
   <tableColumns count="5">
     <tableColumn id="9" name="Informe"/>
     <tableColumn id="10" name="Filtro"/>
@@ -1300,7 +1300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Inasistencias por curso</t>
+          <t>Detalle actualizado matrículas</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -1433,17 +1433,17 @@
       <c r="G6" s="6" t="n"/>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Inasistencias por curso</t>
+          <t>Detalle actualizado matrículas</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Sede - jornada</t>
+          <t>Período</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>B2G - Única</t>
+          <t>B2G_YES BOGOTA-2 C1_SEP_2026</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -1471,17 +1471,17 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Inasistencias por curso</t>
+          <t>Detalle actualizado matrículas</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Programa</t>
+          <t>Sede - jornada</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>YES BOGOTA 2026-2</t>
+          <t>B2G - Única</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -1509,17 +1509,17 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Inasistencias por curso</t>
+          <t>Detalle actualizado matrículas</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Período</t>
+          <t>Programa</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>B2G_YES BOGOTA-2 C1_SEP_2026</t>
+          <t>YES BOGOTA 2026-2</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -1543,17 +1543,17 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Inasistencias por curso</t>
+          <t>Detalle actualizado matrículas</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Curso</t>
+          <t>¿Incluir cursos archivados?</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1577,17 +1577,17 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Inasistencias por curso</t>
+          <t>Detalle actualizado matrículas</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Formato</t>
+          <t>Curso</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>XLSX</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1609,6 +1609,50 @@
           <t>Vacío = guardar la tabla en CSV. 'Usuarios' = bajar los usuarios de cada curso.</t>
         </is>
       </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Detalle actualizado matrículas</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Formato</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>XLSX</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Detalle actualizado matrículas</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Destino</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>C:/Users/sebastian.mendez/OneDrive - CENTRO COLOMBO AMERICANO/Escritorio/Automatizacion Oxford/Descargas/Q10</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>